<commit_message>
Products: refresh catalog from updated Product.xlsx (13 items)
- Regenerate products.json from the revised Excel: new croissant lineup and
  updated prices (plain NT$80; croissants NT$135–150; danish NT$550/600;
  gifts NT$550/680)
- Add en/ja/ko translations + clean slug ids for the five new croissants
  (lemon, honey-longan, black-sesame, sunset salted-yolk, rose-raspberry)
- Refresh product photos; remove images for discontinued items so the folder
  matches the catalogue exactly (13)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Doc/Product.xlsx
+++ b/Doc/Product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/46313b10c5ab42cf/文件/Claude/Projects/Bakery_Website/Doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="11_AD4DBB64A54DDB1B405E38481D5B2C8F4F90DF24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBAC467A-6F88-4161-9A6A-AF26E8694979}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="11_AD4DBB64A54DDB1B405E38481D5B2C8F4F90DF24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3AB3BF3-40A0-41FB-8061-A69F3ECE6CE0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
   <si>
     <t>主標題</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -47,157 +47,153 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>酒精</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>無</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>有</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>說明</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>茶香龍眼丹麥棒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>丹麥油條棒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>丹麥棒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>特色禮盒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>夕陽金沙夾心餅</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>台灣鳳梨酥</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>signature-danish-youtiao.jpg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>S__17506335.jpg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gift.jpg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>800x.jpg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>茶香伴風景，甜在旅程</t>
+  </si>
+  <si>
+    <t>熟悉記憶，優雅重逢</t>
+  </si>
+  <si>
+    <t>把淡水夕陽帶回家</t>
+  </si>
+  <si>
+    <t>將台灣風味細細珍藏</t>
+  </si>
+  <si>
     <t>原味可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>開心果可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>檸檬可頌</t>
   </si>
   <si>
     <t>巧克力可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>蜜香龍眼可頌</t>
+  </si>
+  <si>
+    <t>抹茶可頌</t>
+  </si>
+  <si>
+    <t>黑芝麻可頌</t>
+  </si>
+  <si>
+    <t>夕陽金沙可頌</t>
   </si>
   <si>
     <t>提拉米蘇可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>酒精</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>無</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>有</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Product(2).jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Product(3).jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Product(4).jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Product(5).jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>抹茶可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>金沙可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>玫瑰可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Product(6).jpg</t>
-  </si>
-  <si>
-    <t>Product(7).jpg</t>
-  </si>
-  <si>
-    <t>Product(8).jpg</t>
-  </si>
-  <si>
-    <t>Product(1).jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>說明</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>一切美好，從奶香開始</t>
-  </si>
-  <si>
-    <t>花開時，香氣剛剛好</t>
-  </si>
-  <si>
-    <t>濃郁，是最溫柔的答案</t>
-  </si>
-  <si>
-    <t>微醺一口，時光慢了些</t>
-  </si>
-  <si>
-    <t>靜靜品味，一抹茶香</t>
-  </si>
-  <si>
-    <t>鹹香之中，藏著驚喜</t>
-  </si>
-  <si>
-    <t>每一口，都值得珍藏</t>
-  </si>
-  <si>
-    <t>冰涼與酥香的邂逅</t>
-  </si>
-  <si>
-    <t>台灣古早冰可頌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>茶香龍眼丹麥棒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>丹麥油條棒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>丹麥棒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>特色禮盒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>夕陽金沙夾心餅</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>台灣鳳梨酥</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>signature-danish-youtiao.jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>S__17506335.jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Gift.jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>800x.jpg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>茶香伴風景，甜在旅程</t>
-  </si>
-  <si>
-    <t>熟悉記憶，優雅重逢</t>
-  </si>
-  <si>
-    <t>把淡水夕陽帶回家</t>
-  </si>
-  <si>
-    <t>將台灣風味細細珍藏</t>
+  </si>
+  <si>
+    <t>玫瑰覆盆子可頌</t>
+  </si>
+  <si>
+    <t>圖片1.jpg</t>
+  </si>
+  <si>
+    <t>圖片2.jpg</t>
+  </si>
+  <si>
+    <t>圖片3.jpg</t>
+  </si>
+  <si>
+    <t>圖片4.jpg</t>
+  </si>
+  <si>
+    <t>圖片5.jpg</t>
+  </si>
+  <si>
+    <t>圖片6.jpg</t>
+  </si>
+  <si>
+    <t>圖片7.jpg</t>
+  </si>
+  <si>
+    <t>圖片8.jpg</t>
+  </si>
+  <si>
+    <t>圖片9.jpg</t>
+  </si>
+  <si>
+    <t>奶香，是旅程的開始</t>
+  </si>
+  <si>
+    <t>晨光般的清新酸香</t>
+  </si>
+  <si>
+    <t>深邃可可，靜靜綻放</t>
+  </si>
+  <si>
+    <t>蜜香流轉，餘韻悠長</t>
+  </si>
+  <si>
+    <t>一抹茶韻，靜心回甘</t>
+  </si>
+  <si>
+    <t>芝麻醇厚，溫柔留香</t>
+  </si>
+  <si>
+    <t>把夕陽烘進每一口</t>
+  </si>
+  <si>
+    <t>微醺可可，慢享時光</t>
+  </si>
+  <si>
+    <t>花果芬芳，浪漫盛放</t>
   </si>
 </sst>
 </file>
@@ -207,7 +203,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="&quot;NT$&quot;#,##0_);\(&quot;NT$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +215,15 @@
       <sz val="9"/>
       <name val="新細明體"/>
       <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
@@ -243,9 +248,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -530,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -549,10 +560,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -566,19 +577,19 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -586,19 +597,19 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E3" s="1">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -606,19 +617,19 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E4" s="1">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -626,19 +637,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E5" s="1">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -646,19 +657,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E6" s="1">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -666,19 +677,19 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E7" s="1">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -686,19 +697,19 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E8" s="1">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -706,36 +717,36 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E9" s="1">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F9" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>43</v>
+        <v>31</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E10" s="1">
-        <v>380</v>
+        <v>150</v>
       </c>
       <c r="F10" t="s">
         <v>40</v>
@@ -743,63 +754,123 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E11" s="1">
-        <v>380</v>
+        <v>550</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1">
-        <v>520</v>
+        <v>600</v>
       </c>
       <c r="F12" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E13" s="1">
-        <v>640</v>
+        <v>550</v>
       </c>
       <c r="F13" t="s">
-        <v>42</v>
-      </c>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="1">
+        <v>680</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+    </row>
+    <row r="27" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>